<commit_message>
Deploying to gh-pages from  @ 8d2ee5ac4c06b2044b59eeddc40b5313dee9ef6d 🚀
</commit_message>
<xml_diff>
--- a/en/data/scripts/excel/sdg-data-formatado.xlsx
+++ b/en/data/scripts/excel/sdg-data-formatado.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -753,6 +753,23 @@
       <c r="F16" s="2" t="n"/>
       <c r="G16" s="2" t="n"/>
     </row>
+    <row r="17" ht="25" customHeight="1">
+      <c r="A17" s="2" t="n">
+        <v>2018</v>
+      </c>
+      <c r="B17" s="2" t="inlineStr"/>
+      <c r="C17" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="n"/>
+      <c r="F17" s="2" t="n"/>
+      <c r="G17" s="2" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
Deploying to gh-pages from  @ d6f96ded2994ca1112160b101b92781d0b5c4a5f 🚀
</commit_message>
<xml_diff>
--- a/en/data/scripts/excel/sdg-data-formatado.xlsx
+++ b/en/data/scripts/excel/sdg-data-formatado.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -770,6 +770,23 @@
       <c r="F17" s="2" t="n"/>
       <c r="G17" s="2" t="n"/>
     </row>
+    <row r="18" ht="25" customHeight="1">
+      <c r="A18" s="2" t="n">
+        <v>2019</v>
+      </c>
+      <c r="B18" s="2" t="inlineStr"/>
+      <c r="C18" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="n"/>
+      <c r="F18" s="2" t="n"/>
+      <c r="G18" s="2" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
Deploying to gh-pages from  @ 2d248ce5f39001b8d8ed74c4864fd9d482191e2c 🚀
</commit_message>
<xml_diff>
--- a/en/data/scripts/excel/sdg-data-formatado.xlsx
+++ b/en/data/scripts/excel/sdg-data-formatado.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="indicator" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SDG1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -27,9 +27,6 @@
     </font>
     <font>
       <b val="1"/>
-    </font>
-    <font>
-      <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="14"/>
     </font>
@@ -37,8 +34,11 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
     </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -49,6 +49,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00FF0000"/>
         <bgColor rgb="00FF0000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E0E0E0"/>
+        <bgColor rgb="00E0E0E0"/>
       </patternFill>
     </fill>
   </fills>
@@ -72,16 +78,14 @@
   </cellStyleXfs>
   <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -447,11 +451,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
     <col width="50" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
@@ -462,7 +466,7 @@
     <row r="1" ht="25" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>SDGindicator: indicator</t>
+          <t>SDG1: Sustainable Development Goal 1</t>
         </is>
       </c>
       <c r="B1" s="2" t="n"/>
@@ -514,278 +518,479 @@
     <row r="3" ht="25" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>Year</t>
+          <t>Metric</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>Semestre</t>
+          <t>1.1</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>Value</t>
-        </is>
-      </c>
-      <c r="D3" s="4" t="inlineStr">
-        <is>
-          <t>Group</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="n"/>
-      <c r="F3" s="2" t="n"/>
-      <c r="G3" s="2" t="n"/>
+          <t>Metric 1.1</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="n"/>
+      <c r="E3" s="4" t="n"/>
+      <c r="F3" s="4" t="n"/>
+      <c r="G3" s="4" t="n"/>
     </row>
     <row r="4" ht="25" customHeight="1">
-      <c r="A4" s="2" t="n">
-        <v>2025</v>
-      </c>
-      <c r="B4" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C4" s="2" t="n">
-        <v>60</v>
-      </c>
-      <c r="D4" s="2" t="inlineStr"/>
-      <c r="E4" s="2" t="n"/>
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Indicator</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>2015</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="F4" s="2" t="n"/>
       <c r="G4" s="2" t="n"/>
     </row>
     <row r="5" ht="25" customHeight="1">
-      <c r="A5" s="2" t="n">
-        <v>2025</v>
-      </c>
-      <c r="B5" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="C5" s="2" t="n">
-        <v>50</v>
-      </c>
-      <c r="D5" s="2" t="inlineStr"/>
-      <c r="E5" s="2" t="n"/>
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Indicator</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>2015</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="F5" s="2" t="n"/>
       <c r="G5" s="2" t="n"/>
     </row>
     <row r="6" ht="25" customHeight="1">
-      <c r="A6" s="2" t="n">
-        <v>2015</v>
-      </c>
-      <c r="B6" s="2" t="inlineStr"/>
-      <c r="C6" s="2" t="n">
-        <v>1</v>
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Indicator</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>2015</t>
+        </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="n"/>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="F6" s="2" t="n"/>
       <c r="G6" s="2" t="n"/>
     </row>
     <row r="7" ht="25" customHeight="1">
-      <c r="A7" s="2" t="n">
-        <v>2015</v>
-      </c>
-      <c r="B7" s="2" t="inlineStr"/>
-      <c r="C7" s="2" t="n">
-        <v>3</v>
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Indicator</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>2016</t>
+        </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="n"/>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="F7" s="2" t="n"/>
       <c r="G7" s="2" t="n"/>
     </row>
     <row r="8" ht="25" customHeight="1">
-      <c r="A8" s="2" t="n">
-        <v>2015</v>
-      </c>
-      <c r="B8" s="2" t="inlineStr"/>
-      <c r="C8" s="2" t="n">
-        <v>2</v>
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Indicator</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>2016</t>
+        </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="n"/>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="F8" s="2" t="n"/>
       <c r="G8" s="2" t="n"/>
     </row>
     <row r="9" ht="25" customHeight="1">
-      <c r="A9" s="2" t="n">
-        <v>2016</v>
-      </c>
-      <c r="B9" s="2" t="inlineStr"/>
-      <c r="C9" s="2" t="n">
-        <v>1</v>
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Indicator</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>2016</t>
+        </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="n"/>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="F9" s="2" t="n"/>
       <c r="G9" s="2" t="n"/>
     </row>
     <row r="10" ht="25" customHeight="1">
-      <c r="A10" s="2" t="n">
-        <v>2016</v>
-      </c>
-      <c r="B10" s="2" t="inlineStr"/>
-      <c r="C10" s="2" t="n">
-        <v>3</v>
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Indicator</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>2017</t>
+        </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="n"/>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="F10" s="2" t="n"/>
       <c r="G10" s="2" t="n"/>
     </row>
     <row r="11" ht="25" customHeight="1">
-      <c r="A11" s="2" t="n">
-        <v>2016</v>
-      </c>
-      <c r="B11" s="2" t="inlineStr"/>
-      <c r="C11" s="2" t="n">
-        <v>2</v>
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Indicator</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>2017</t>
+        </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="n"/>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="F11" s="2" t="n"/>
       <c r="G11" s="2" t="n"/>
     </row>
     <row r="12" ht="25" customHeight="1">
-      <c r="A12" s="2" t="n">
-        <v>2017</v>
-      </c>
-      <c r="B12" s="2" t="inlineStr"/>
-      <c r="C12" s="2" t="n">
-        <v>3</v>
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Indicator</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>2017</t>
+        </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="n"/>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="F12" s="2" t="n"/>
       <c r="G12" s="2" t="n"/>
     </row>
     <row r="13" ht="25" customHeight="1">
-      <c r="A13" s="2" t="n">
-        <v>2017</v>
-      </c>
-      <c r="B13" s="2" t="inlineStr"/>
-      <c r="C13" s="2" t="n">
-        <v>1</v>
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Indicator</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>2018</t>
+        </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="n"/>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="F13" s="2" t="n"/>
       <c r="G13" s="2" t="n"/>
     </row>
     <row r="14" ht="25" customHeight="1">
-      <c r="A14" s="2" t="n">
-        <v>2017</v>
-      </c>
-      <c r="B14" s="2" t="inlineStr"/>
-      <c r="C14" s="2" t="n">
-        <v>2</v>
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Indicator</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>2018</t>
+        </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="n"/>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="F14" s="2" t="n"/>
       <c r="G14" s="2" t="n"/>
     </row>
     <row r="15" ht="25" customHeight="1">
-      <c r="A15" s="2" t="n">
-        <v>2018</v>
-      </c>
-      <c r="B15" s="2" t="inlineStr"/>
-      <c r="C15" s="2" t="n">
-        <v>1</v>
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Indicator</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>2018</t>
+        </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="E15" s="2" t="n"/>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="F15" s="2" t="n"/>
       <c r="G15" s="2" t="n"/>
     </row>
     <row r="16" ht="25" customHeight="1">
-      <c r="A16" s="2" t="n">
-        <v>2018</v>
-      </c>
-      <c r="B16" s="2" t="inlineStr"/>
-      <c r="C16" s="2" t="n">
-        <v>2</v>
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Indicator</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="n"/>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
       <c r="F16" s="2" t="n"/>
       <c r="G16" s="2" t="n"/>
     </row>
     <row r="17" ht="25" customHeight="1">
-      <c r="A17" s="2" t="n">
-        <v>2018</v>
-      </c>
-      <c r="B17" s="2" t="inlineStr"/>
-      <c r="C17" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="E17" s="2" t="n"/>
-      <c r="F17" s="2" t="n"/>
-      <c r="G17" s="2" t="n"/>
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>Metric 1.2</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="n"/>
+      <c r="E17" s="4" t="n"/>
+      <c r="F17" s="4" t="n"/>
+      <c r="G17" s="4" t="n"/>
     </row>
     <row r="18" ht="25" customHeight="1">
-      <c r="A18" s="2" t="n">
-        <v>2019</v>
-      </c>
-      <c r="B18" s="2" t="inlineStr"/>
-      <c r="C18" s="2" t="n">
-        <v>4</v>
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Indicator</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>1.2.2</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="n"/>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
       <c r="F18" s="2" t="n"/>
       <c r="G18" s="2" t="n"/>
+    </row>
+    <row r="19" ht="25" customHeight="1">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Indicator</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>1.2.2</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="n"/>
+      <c r="G19" s="2" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
Deploying to gh-pages from  @ 361f3a947101c1d2de6d969d718df63420059201 🚀
</commit_message>
<xml_diff>
--- a/en/data/scripts/excel/sdg-data-formatado.xlsx
+++ b/en/data/scripts/excel/sdg-data-formatado.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SDG1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SDG5" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -998,4 +999,161 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="50" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="25" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>SDG5: Sustainable Development Goal 5</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="2" t="n"/>
+      <c r="D1" s="2" t="n"/>
+      <c r="E1" s="2" t="n"/>
+      <c r="F1" s="2" t="n"/>
+      <c r="G1" s="2" t="n"/>
+    </row>
+    <row r="2" ht="25" customHeight="1">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Metric and indicator reference</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Metric / Indicator</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>Value
+(for continuous data)</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>Yes/No</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>Evidence</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>Public
+(Yes/No)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="25" customHeight="1">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>5.1</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Metric 5.1</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="n"/>
+      <c r="E3" s="4" t="n"/>
+      <c r="F3" s="4" t="n"/>
+      <c r="G3" s="4" t="n"/>
+    </row>
+    <row r="4" ht="25" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Indicator</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>5.1.1</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>2017</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="n"/>
+      <c r="G4" s="2" t="n"/>
+    </row>
+    <row r="5" ht="25" customHeight="1">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Indicator</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>5.1.1</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="n"/>
+      <c r="G5" s="2" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:G1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>